<commit_message>
🎯 Strike: mono_other upload re-split into 8 files of ≤200
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brand-protection/2026-09-28/strike/01-mono_other-p4.xlsx
+++ b/brand-protection/2026-09-28/strike/01-mono_other-p4.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M84"/>
+  <dimension ref="A1:M201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://up-space.ru/</t>
+          <t>https://mostbet-azerbaijan-fun.org/</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -499,21 +499,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>up-space.ru</t>
+          <t>mostbet-azerbaijan-fun.org</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://urbanofficearchitecture.com/</t>
+          <t>https://mostbet-azerbaijan-game.com/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -533,14 +528,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>urbanofficearchitecture.com</t>
+          <t>mostbet-azerbaijan-game.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://urfolab.ru/</t>
+          <t>https://mostbet-azerbaijan-games.com/</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -555,19 +550,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>urfolab.ru</t>
+          <t>mostbet-azerbaijan-games.com</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://urperm.ru/</t>
+          <t>https://mostbet-azerbaijan-jackpot.com/</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -582,19 +577,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>urperm.ru</t>
+          <t>mostbet-azerbaijan-jackpot.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://uz-mostbet-apk.com/</t>
+          <t>https://mostbet-azerbaijan-jackpot.net/</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -607,21 +602,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>uz-mostbet-apk.com</t>
+          <t>mostbet-azerbaijan-jackpot.net</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://uz-mostbet-skachat.com/</t>
+          <t>https://mostbet-azerbaijan-jackpot.org/</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -634,21 +624,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>uz-mostbet-skachat.com</t>
+          <t>mostbet-azerbaijan-jackpot.org</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://uz-mostbet.bet/</t>
+          <t>https://mostbet-azerbaijan-max.net/</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -663,14 +648,14 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>uz-mostbet.bet</t>
+          <t>mostbet-azerbaijan-max.net</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://uz-mostbets.com/</t>
+          <t>https://mostbet-azerbaijan-play.net/</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -683,21 +668,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>uz-mostbets.com</t>
+          <t>mostbet-azerbaijan-play.net</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://uzbekmarket.ru/</t>
+          <t>https://mostbet-azerbaijan-pro.net/</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -710,21 +690,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>uzbekmarket.ru</t>
+          <t>mostbet-azerbaijan-pro.net</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://uzbet-mostbet.com/</t>
+          <t>https://mostbet-azerbaijan-sport.com/</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -744,14 +719,14 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>uzbet-mostbet.com</t>
+          <t>mostbet-azerbaijan-sport.com</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://uzbet-mostbet.ink/</t>
+          <t>https://mostbet-azerbaijan-sport.net/</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -766,14 +741,14 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>uzbet-mostbet.ink</t>
+          <t>mostbet-azerbaijan-sport.net</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://uzmostbet-kirish.com/</t>
+          <t>https://mostbet-azerbaijan-sport.org/</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -786,21 +761,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>uzmostbet-kirish.com</t>
+          <t>mostbet-azerbaijan-sport.org</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://uzmostbetskachat.com/</t>
+          <t>https://mostbet-azerbaijan-vip.com/</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -820,14 +790,14 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>uzmostbetskachat.com</t>
+          <t>mostbet-azerbaijan-vip.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://vangoghlife.ru/</t>
+          <t>https://mostbet-azerbaijan-win.net/</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -840,21 +810,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>vangoghlife.ru</t>
+          <t>mostbet-azerbaijan-win.net</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://veda-inform.ru/</t>
+          <t>https://mostbet-azerbaijan.org/</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -867,21 +832,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>veda-inform.ru</t>
+          <t>mostbet-azerbaijan.org</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://veganationmtl.com/</t>
+          <t>https://mostbet-azerbaycan.fun/</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -894,21 +854,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>veganationmtl.com</t>
+          <t>mostbet-azerbaycan.fun</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://velopolosa.ru/</t>
+          <t>https://mostbet-azz.ink/</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -921,21 +876,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>velopolosa.ru</t>
+          <t>mostbet-azz.ink</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://venetianartssociety.org/</t>
+          <t>https://mostbet-bd-casino.biz/</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -950,14 +900,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>venetianartssociety.org</t>
+          <t>mostbet-bd-casino.biz</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://vesta34.ru/</t>
+          <t>https://mostbet-bd.cloud/</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -970,21 +920,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>vesta34.ru</t>
+          <t>mostbet-bd.cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://viaexpert.pl/</t>
+          <t>https://mostbet-bd.digital/</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -997,21 +942,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>viaexpert.pl</t>
+          <t>mostbet-bd.digital</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://viapublication.com/</t>
+          <t>https://mostbet-bd.icu/</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1024,21 +964,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>viapublication.com</t>
+          <t>mostbet-bd.icu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://viapublicationcom.click/</t>
+          <t>https://mostbet-bd.pro/</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1053,14 +988,14 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>viapublicationcom.click</t>
+          <t>mostbet-bd.pro</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://vigvamkids.ru/</t>
+          <t>https://mostbet-bd.space/</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1073,21 +1008,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>vigvamkids.ru</t>
+          <t>mostbet-bd.space</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://virginiabeachrockgym.com/</t>
+          <t>https://mostbet-best.org/</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1100,21 +1030,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>virginiabeachrockgym.com</t>
+          <t>mostbet-best.org</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://visitbar.org/</t>
+          <t>https://mostbet-bet.org/</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1129,14 +1054,14 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>visitbar.org</t>
+          <t>mostbet-bet.org</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://vivasan-rus.ru/</t>
+          <t>https://mostbet-bonus-play.com/</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1151,19 +1076,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>vivasan-rus.ru</t>
+          <t>mostbet-bonus-play.com</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://vlc.vin/</t>
+          <t>https://mostbet-bookmakers.ru/</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1176,16 +1101,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>vlc.vin</t>
+          <t>mostbet-bookmakers.ru</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://vm-energy.ru/</t>
+          <t>https://mostbet-brand-pl.best/</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1198,21 +1128,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>vm-energy.ru</t>
+          <t>mostbet-brand-pl.best</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://vofelysandor.hu/</t>
+          <t>https://mostbet-brand-pl.click/</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1225,21 +1150,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>HU</t>
-        </is>
-      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>vofelysandor.hu</t>
+          <t>mostbet-brand-pl.click</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://voices-festival.org/</t>
+          <t>https://mostbet-brand-pl.com/</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1252,16 +1172,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>voices-festival.org</t>
+          <t>mostbet-brand-pl.com</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://voicesfestival.click/</t>
+          <t>https://mostbet-brand.pro/</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1276,14 +1201,14 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>voicesfestival.click</t>
+          <t>mostbet-brand.pro</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://vokalme.ru/</t>
+          <t>https://mostbet-bukmeker-kontoru.top/</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1296,21 +1221,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>vokalme.ru</t>
+          <t>mostbet-bukmeker-kontoru.top</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://voronezh-haval.ru/</t>
+          <t>https://mostbet-casino-2025.pl/</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1325,19 +1245,19 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>voronezh-haval.ru</t>
+          <t>mostbet-casino-2025.pl</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://vp-clinic.ru/</t>
+          <t>https://mostbet-casino-app.ru/</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1357,14 +1277,14 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>vp-clinic.ru</t>
+          <t>mostbet-casino-app.ru</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://vseprintera.ru/</t>
+          <t>https://mostbet-casino-azerbaijan.com/</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1379,19 +1299,19 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>vseprintera.ru</t>
+          <t>mostbet-casino-azerbaijan.com</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://vsetkani.cfd/</t>
+          <t>https://mostbet-casino-azerbaijan.net/</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1406,14 +1326,14 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>vsetkani.cfd</t>
+          <t>mostbet-casino-azerbaijan.net</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://vsetkani.info/</t>
+          <t>https://mostbet-casino-azerbaijan.org/</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1428,14 +1348,14 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>vsetkani.info</t>
+          <t>mostbet-casino-azerbaijan.org</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://wallclub.ru/</t>
+          <t>https://mostbet-casino-bet-az.com/</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1450,19 +1370,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>wallclub.ru</t>
+          <t>mostbet-casino-bet-az.com</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://warriorsteam.pl/</t>
+          <t>https://mostbet-casino-bonus.com.de/</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1477,19 +1397,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>warriorsteam.pl</t>
+          <t>mostbet-casino-bonus.com.de</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://waterapps.net/</t>
+          <t>https://mostbet-casino-com.pl/</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1502,16 +1422,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>waterapps.net</t>
+          <t>mostbet-casino-com.pl</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://wcflcr2017.com/</t>
+          <t>https://mostbet-casino-cz.org/</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1524,21 +1449,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>wcflcr2017.com</t>
+          <t>mostbet-casino-cz.org</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://wcftutorial.net/</t>
+          <t>https://mostbet-casino-czechia.cz/</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1551,16 +1471,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>wcftutorial.net</t>
+          <t>mostbet-casino-czechia.cz</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://webmayak.pro/</t>
+          <t>https://mostbet-casino-es.top/</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1575,14 +1500,14 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>webmayak.pro</t>
+          <t>mostbet-casino-es.top</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://wildhorsewebworks.com/</t>
+          <t>https://mostbet-casino-game.net/</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1595,21 +1520,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>wildhorsewebworks.com</t>
+          <t>mostbet-casino-game.net</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://winterhockeygames.com/</t>
+          <t>https://mostbet-casino-gr.com/</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1629,14 +1549,14 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>winterhockeygames.com</t>
+          <t>mostbet-casino-gr.com</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://worldofphotos.ru/</t>
+          <t>https://mostbet-casino-kasyno.pl/</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1651,19 +1571,19 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>worldofphotos.ru</t>
+          <t>mostbet-casino-kasyno.pl</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://wwwantigeliru.top/</t>
+          <t>https://mostbet-casino-login.com/</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1676,16 +1596,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>wwwantigeliru.top</t>
+          <t>mostbet-casino-login.com</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://wwwnbspolicyplatformorg.top/</t>
+          <t>https://mostbet-casino-mirror-3.cfd/</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1700,14 +1625,14 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>wwwnbspolicyplatformorg.top</t>
+          <t>mostbet-casino-mirror-3.cfd</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://wwwtehregru.cfd/</t>
+          <t>https://mostbet-casino-nl.com/</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1720,16 +1645,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>wwwtehregru.cfd</t>
+          <t>mostbet-casino-nl.com</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://wwwtehregru1.cfd/</t>
+          <t>https://mostbet-casino-no.com/</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1742,16 +1672,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>wwwtehregru1.cfd</t>
+          <t>mostbet-casino-no.com</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://wwwtehregru2.cfd/</t>
+          <t>https://mostbet-casino-nz.com/</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1764,16 +1699,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>wwwtehregru2.cfd</t>
+          <t>mostbet-casino-nz.com</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://wwwtelepartypro.xyz/</t>
+          <t>https://mostbet-casino-ofb.fun/</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1788,14 +1728,14 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>wwwtelepartypro.xyz</t>
+          <t>mostbet-casino-ofb.fun</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://xldb.org/</t>
+          <t>https://mostbet-casino-online-cz.cz/</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1808,16 +1748,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>xldb.org</t>
+          <t>mostbet-casino-online-cz.cz</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://xn----7sbajchefi3c5abkjc2d4i.xn--p1ai/</t>
+          <t>https://mostbet-casino-online-cz.eu.com/</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1830,16 +1775,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>фаергард-поволжье.рф</t>
+          <t>mostbet-casino-online-cz.eu.com</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://xn----7sblece8bdveh9l.xn--p1ai/</t>
+          <t>https://mostbet-casino-online.com/</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1852,16 +1802,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>дренаж-пермь.рф</t>
+          <t>mostbet-casino-online.com</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://xn----7sbqgez1bcecc.xn--p1ai/</t>
+          <t>https://mostbet-casino-online.net/</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1876,14 +1831,14 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>аутизм-тест.рф</t>
+          <t>mostbet-casino-online.net</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://xn----8sba7blnqd3a.xn--p1ai/</t>
+          <t>https://mostbet-casino-online.pt/</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1896,16 +1851,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>рц-атлант.рф</t>
+          <t>mostbet-casino-online.pt</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://xn----ctbbmvm0c3a2c.xn--p1ai/</t>
+          <t>https://mostbet-casino-online.win/</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1920,14 +1880,14 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>кмв-цветы.рф</t>
+          <t>mostbet-casino-online.win</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://xn----dtbfea6a0akik4e6a9a.xn--p1ai/</t>
+          <t>https://mostbet-casino-pt.bet/</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1942,14 +1902,14 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>люстры-дешево.рф</t>
+          <t>mostbet-casino-pt.bet</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://xn--80aaah0dhi.xn--p1ai/</t>
+          <t>https://mostbet-casino-pt.org/</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1964,14 +1924,14 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>параван.рф</t>
+          <t>mostbet-casino-pt.org</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://xn--80aabbgg8aaod1ahg0k3e.xn--p1ai/</t>
+          <t>https://mostbet-casino-qtr2.ru/</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1984,16 +1944,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>банябочкавикинг.рф</t>
+          <t>mostbet-casino-qtr2.ru</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://xn--80abcf9dqr.xn--p1ai/</t>
+          <t>https://mostbet-casino-qtr3.ru/</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2006,16 +1971,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>вбуграх.рф</t>
+          <t>mostbet-casino-qtr3.ru</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://xn--80ahbnxidcjb.xn--p1ai/</t>
+          <t>https://mostbet-casino-ro.ro/</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2028,16 +1998,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>природадом.рф</t>
+          <t>mostbet-casino-ro.ro</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://xn--80ahklijc.xn--p1ai/</t>
+          <t>https://mostbet-casino-romania.ro/</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2050,16 +2025,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>домакзн.рф</t>
+          <t>mostbet-casino-romania.ro</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://xn--90ahpcrbldgh1j.xn--p1ai/</t>
+          <t>https://mostbet-casino-tajikistan.com/</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2072,16 +2052,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>электросбор.рф</t>
+          <t>mostbet-casino-tajikistan.com</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://xn--90aitipgc.net/</t>
+          <t>https://mostbet-casino-uk.com/</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2094,16 +2079,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>мостбет.net</t>
+          <t>mostbet-casino-uk.com</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://xn--90aitipgc.su/</t>
+          <t>https://mostbet-casino-ux4.ru/</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2116,16 +2106,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>мостбет.su</t>
+          <t>mostbet-casino-ux4.ru</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://yanevestachita.ru/</t>
+          <t>https://mostbet-casino-uz.com/</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2140,19 +2135,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>yanevestachita.ru</t>
+          <t>mostbet-casino-uz.com</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://yeahstub.com/</t>
+          <t>https://mostbet-casino-uz.net/</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2165,21 +2160,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>yeahstub.com</t>
+          <t>mostbet-casino-uz.net</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://yeehawindustries.com/</t>
+          <t>https://mostbet-casino-uz.org/</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2192,21 +2182,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>yeehawindustries.com</t>
+          <t>mostbet-casino-uz.org</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://yi-fighting.ru/</t>
+          <t>https://mostbet-casino-uzbekistan.com/</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2221,19 +2206,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>yi-fighting.ru</t>
+          <t>mostbet-casino-uzbekistan.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://yoheim-eda.ru/</t>
+          <t>https://mostbet-casino-yeh.buzz/</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2246,21 +2231,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>yoheim-eda.ru</t>
+          <t>mostbet-casino-yeh.buzz</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://yuliafotoskazka.ru/</t>
+          <t>https://mostbet-casino-zd5.ru/</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2280,14 +2260,14 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>yuliafotoskazka.ru</t>
+          <t>mostbet-casino-zd5.ru</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://zagorodnii-mir.ru/</t>
+          <t>https://mostbet-casino.biz.pl/</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2302,19 +2282,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>zagorodnii-mir.ru</t>
+          <t>mostbet-casino.biz.pl</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://zappgum.com/</t>
+          <t>https://mostbet-casino.click/</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2327,21 +2307,16 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>zappgum.com</t>
+          <t>mostbet-casino.click</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://zarzadzanieit.com/</t>
+          <t>https://mostbet-casino.com.co/</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2356,19 +2331,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>zarzadzanieit.com</t>
+          <t>mostbet-casino.com.co</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://zerkalo-mostbet-one.com/</t>
+          <t>https://mostbet-casino.info.pl/</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2383,19 +2358,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>zerkalo-mostbet-one.com</t>
+          <t>mostbet-casino.info.pl</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://zgm.mn/</t>
+          <t>https://mostbet-casino1.com/</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2410,19 +2385,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>zgm.mn</t>
+          <t>mostbet-casino1.com</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://zhasproject-karaganda-kostanai.kz/</t>
+          <t>https://mostbet-casino1.com.pl/</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2437,19 +2412,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>zhasproject-karaganda-kostanai.kz</t>
+          <t>mostbet-casino1.com.pl</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://zhasprojectkaragandakostanaikz.cfd/</t>
+          <t>https://mostbet-casino1.pl/</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2462,16 +2437,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>zhasprojectkaragandakostanaikz.cfd</t>
+          <t>mostbet-casino1.pl</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://zielonakuchnia.eu/</t>
+          <t>https://mostbet-casino247.ru/</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2484,16 +2464,21 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>zielonakuchnia.eu</t>
+          <t>mostbet-casino247.ru</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://znanie100.ru/</t>
+          <t>https://mostbet-casinocz.com/</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2508,19 +2493,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>GLOBAL</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>znanie100.ru</t>
+          <t>mostbet-casinocz.com</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://zsstruznice.cz/</t>
+          <t>https://mostbet-casinohu.org/</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2533,14 +2518,2958 @@
           <t>strike-01-mono-other,strike-01-mono-other-p4</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>mostbet-casinohu.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>https://mostbet-casinoindia.com/</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>mostbet-casinoindia.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>https://mostbet-casinos.de/</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>mostbet-casinos.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>https://mostbet-casinoz.cz/</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>zsstruznice.cz</t>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>mostbet-casinoz.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>https://mostbet-cassino-br.com/</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>mostbet-cassino-br.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>https://mostbet-chile.org/</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>mostbet-chile.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>https://mostbet-code.com/</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>mostbet-code.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>https://mostbet-com.com/</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>mostbet-com.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>https://mostbet-crash.kz/</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>KZ</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>mostbet-crash.kz</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>https://mostbet-cz-casino.win/</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>mostbet-cz-casino.win</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>https://mostbet-cz.win/</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>mostbet-cz.win</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>https://mostbet-deutsch-casino.com/</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>mostbet-deutsch-casino.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>https://mostbet-dfg34.com/</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>mostbet-dfg34.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>https://mostbet-fgh48.com/</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>mostbet-fgh48.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>https://mostbet-france.com/</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>mostbet-france.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>https://mostbet-gamble.com/</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>mostbet-gamble.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>https://mostbet-gambling.net/</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>mostbet-gambling.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>https://mostbet-game-az.com/</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>mostbet-game-az.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>https://mostbet-game.org/</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>mostbet-game.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>https://mostbet-gaming-play.com/</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>mostbet-gaming-play.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>https://mostbet-gaming.net/</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>mostbet-gaming.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>https://mostbet-gaming.org/</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>mostbet-gaming.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>https://mostbet-ghj15.com/</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>mostbet-ghj15.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>https://mostbet-giris-tr.net/</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>mostbet-giris-tr.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>https://mostbet-giriss.ink/</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>mostbet-giriss.ink</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>https://mostbet-hesab.com/</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>mostbet-hesab.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>https://mostbet-hu.it.com/</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>mostbet-hu.it.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>https://mostbet-hu.win/</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>mostbet-hu.win</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>https://mostbet-hu3.com/</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>mostbet-hu3.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>https://mostbet-hu4.com/</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>mostbet-hu4.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>https://mostbet-hu5.com/</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>mostbet-hu5.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>https://mostbet-hun.jp.net/</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>mostbet-hun.jp.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>https://mostbet-hungary.app/</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>mostbet-hungary.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>https://mostbet-igambling.com/</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>mostbet-igambling.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>https://mostbet-in.org/</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>mostbet-in.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>https://mostbet-in.site/</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>mostbet-in.site</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>https://mostbet-ios.com/</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>mostbet-ios.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>https://mostbet-ios.org/</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>mostbet-ios.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>https://mostbet-jackpot.kz/</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>KZ</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>mostbet-jackpot.kz</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>https://mostbet-kasina.cz/</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>mostbet-kasina.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>https://mostbet-kasyno-gra.pl/</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>mostbet-kasyno-gra.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>https://mostbet-kasyno-gracze.pl/</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>mostbet-kasyno-gracze.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>https://mostbet-kasyno-promocja.pl/</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>mostbet-kasyno-promocja.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>https://mostbet-kasyno.com/</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>mostbet-kasyno.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>https://mostbet-kasyno.com.pl/</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>mostbet-kasyno.com.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>https://mostbet-kazino-uz.top/</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>mostbet-kazino-uz.top</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>https://mostbet-kazino-uz1.top/</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>mostbet-kazino-uz1.top</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>https://mostbet-kazino247.ru/</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>mostbet-kazino247.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>https://mostbet-kenya.co.ke/</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>KE</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>mostbet-kenya.co.ke</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>https://mostbet-life-ky.com/</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>mostbet-life-ky.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>https://mostbet-live-bet.com/</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>mostbet-live-bet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>https://mostbet-login-br.com/</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>mostbet-login-br.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>https://mostbet-logowanie.pl/</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>mostbet-logowanie.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobil.net/</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>mostbet-mobil.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobile.net/</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>mostbet-mobile.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobile57-amp.ru/</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>mostbet-mobile57-amp.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobile59-amp.ru/</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>mostbet-mobile59-amp.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobile60-amp.ru/</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>mostbet-mobile60-amp.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobile61-amp.ru/</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>mostbet-mobile61-amp.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobile62-amp.ru/</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>mostbet-mobile62-amp.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>https://mostbet-mobile63-amp.ru/</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>mostbet-mobile63-amp.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>https://mostbet-nederland.com/</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>mostbet-nederland.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>https://mostbet-nl.nl/</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>mostbet-nl.nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>https://mostbet-nz.com/</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>mostbet-nz.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>https://mostbet-offer.com/</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>mostbet-offer.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>https://mostbet-official-az.com/</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>mostbet-official-az.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>https://mostbet-official-pl.com.pl/</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>mostbet-official-pl.com.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>https://mostbet-official-site.fun/</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>mostbet-official-site.fun</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>https://mostbet-officialsite.top/</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>mostbet-officialsite.top</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>https://mostbet-one.net/</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>mostbet-one.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>https://mostbet-online-aplikace.cz/</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>mostbet-online-aplikace.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>https://mostbet-online-bangla.com/</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>mostbet-online-bangla.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>https://mostbet-online-cz.net/</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>mostbet-online-cz.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>https://mostbet-online-game.net/</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>mostbet-online-game.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>https://mostbet-online-game.org/</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>mostbet-online-game.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>https://mostbet-online-kasino.cz/</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>mostbet-online-kasino.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>https://mostbet-online-pt.casino/</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>mostbet-online-pt.casino</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>https://mostbet-online.app/</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>mostbet-online.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>https://mostbet-online.pt/</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>mostbet-online.pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>https://mostbet-onlinetr.top/</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>mostbet-onlinetr.top</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>https://mostbet-pk-casino.org/</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>mostbet-pk-casino.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>https://mostbet-pk.click/</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>mostbet-pk.click</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>https://mostbet-pk.info/</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>mostbet-pk.info</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>https://mostbet-pk.pro/</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>mostbet-pk.pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>https://mostbet-pl-casino-com.pl/</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>mostbet-pl-casino-com.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>https://mostbet-pl.win/</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>mostbet-pl.win</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>https://mostbet-play-online.com/</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>mostbet-play-online.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>https://mostbet-play.cz/</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>mostbet-play.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>https://mostbet-play.org/</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>mostbet-play.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>https://mostbet-play.pl/</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>mostbet-play.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>https://mostbet-playrf.ru/</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>mostbet-playrf.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>https://mostbet-pol.com/</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>mostbet-pol.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>https://mostbet-poland.live/</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>mostbet-poland.live</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>https://mostbet-poland.net.pl/</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>mostbet-poland.net.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>https://mostbet-portu.app/</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>mostbet-portu.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>https://mostbet-portu.pt/</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>mostbet-portu.pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>https://mostbet-portu.site/</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>mostbet-portu.site</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>https://mostbet-portugal.app/</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>mostbet-portugal.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>https://mostbet-portugal.pt/</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>mostbet-portugal.pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>https://mostbet-preimushestva-obzor.ru/</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>mostbet-preimushestva-obzor.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>https://mostbet-promo.kz/</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>KZ</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>mostbet-promo.kz</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>https://mostbet-pt.com.pt/</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>mostbet-pt.com.pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>https://mostbet-rabochee-zerkalo-na-segodnya.ru/</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>mostbet-rabochee-zerkalo-na-segodnya.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>https://mostbet-registrace.cz/</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>mostbet-registrace.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>https://mostbet-review-pt.com/</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>mostbet-review-pt.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>https://mostbet-rfplay.ru/</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>mostbet-rfplay.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>https://mostbet-rg23.com/</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>mostbet-rg23.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>https://mostbet-ro.com.ro/</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>mostbet-ro.com.ro</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>https://mostbet-ro.ro/</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>mostbet-ro.ro</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>https://mostbet-roulette.com/</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>mostbet-roulette.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>https://mostbet-russian.ru/</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>mostbet-russian.ru</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>https://mostbet-schweiz.org/</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>mostbet-schweiz.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>https://mostbet-site-tr.top/</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>mostbet-site-tr.top</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>https://mostbet-site.org/</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>mostbet-site.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>https://mostbet-slot-amp3.top/</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>mostbet-slot-amp3.top</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>https://mostbet-slots-pt.com/</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>mostbet-slots-pt.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>https://mostbet-spin.kz/</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>KZ</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>mostbet-spin.kz</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>https://mostbet-stavka.ru/</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Trademark Infringement</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>strike-01-mono-other,strike-01-mono-other-p4</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>mostbet-stavka.ru</t>
         </is>
       </c>
     </row>

</xml_diff>